<commit_message>
UHG 2027 Drivers: 2026 P1-P10 actual vs P11-P12 forecast side by side
</commit_message>
<xml_diff>
--- a/assets/UHG-Budget-2027.xlsx
+++ b/assets/UHG-Budget-2027.xlsx
@@ -55,10 +55,10 @@
     <numFmt numFmtId="171" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="172" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="173" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="174" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="175" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="174" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0;[Red](&quot;$&quot;#,##0)"/>
   </numFmts>
-  <fonts count="39">
+  <fonts count="47">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -279,8 +279,53 @@
       <color rgb="00E8E0D4"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C9AA7C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00C9AA7C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00E8E0D4"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005A8BA7"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C9AA7C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="005A8BA7"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005A8BA7"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00E8E0D4"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -387,8 +432,13 @@
         <fgColor rgb="000D1620"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003D3420"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="33">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -766,11 +816,25 @@
         <color rgb="003A5060"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="002A3844"/>
+      </left>
+      <right style="thin">
+        <color rgb="002A3844"/>
+      </right>
+      <top style="thin">
+        <color rgb="002A3844"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="002A3844"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="324">
+  <cellXfs count="351">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1312,9 +1376,9 @@
     <xf numFmtId="0" fontId="33" fillId="2" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="175" fontId="35" fillId="19" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="35" fillId="19" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="36" fillId="20" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="175" fontId="36" fillId="20" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="36" fillId="20" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="25" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -1503,6 +1567,47 @@
     <xf numFmtId="170" fontId="24" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="2" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="2" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="2" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="21" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="2" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="44" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="41" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="41" fillId="21" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="39" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="39" fillId="20" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="20" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="41" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="39" fillId="20" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="41" fillId="19" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="39" fillId="20" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="35" fillId="19" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="36" fillId="20" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1580,6 +1685,26 @@
 </file>
 
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>MC</author>
+  </authors>
+  <commentList>
+    <comment ref="A41" authorId="0" shapeId="0">
+      <text>
+        <t>Cloudbeds bookedrevs (else actrevs). 36 keys. P11 = typed $135,000. P12 = file 35% × $190.</t>
+      </text>
+    </comment>
+    <comment ref="A45" authorId="0" shapeId="0">
+      <text>
+        <t>Toast evtrevs FP + 1887. P11–P12 forecast events $0 (file / typed). 2027 events are the $40k/qtr rows above.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>MC</author>
@@ -1898,7 +2023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -1911,6 +2036,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1918,6 +2044,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="216" t="inlineStr">
         <is>
@@ -1932,6 +2059,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="216" t="inlineStr">
         <is>
@@ -1946,6 +2074,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -1953,6 +2082,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -1960,6 +2090,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -1974,6 +2105,26 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="216" t="inlineStr">
+        <is>
+          <t>2026 comparison (13 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Drivers tab now has 2026 P1–P10 actual revenue next to P11–P12 forecast, side by side with the frozen 2027 income row. P13 2026 left blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1986,7 +2137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3121,18 +3272,888 @@
         </is>
       </c>
     </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="324" t="inlineStr">
+        <is>
+          <t>2026 REVENUE vs 2027  ·  P1–P10 actual  ·  P11–P12 forecast</t>
+        </is>
+      </c>
+      <c r="B36" s="325" t="n"/>
+      <c r="C36" s="325" t="n"/>
+      <c r="D36" s="325" t="n"/>
+      <c r="E36" s="325" t="n"/>
+      <c r="F36" s="325" t="n"/>
+      <c r="G36" s="325" t="n"/>
+      <c r="H36" s="325" t="n"/>
+      <c r="I36" s="325" t="n"/>
+      <c r="J36" s="325" t="n"/>
+      <c r="K36" s="325" t="n"/>
+      <c r="L36" s="325" t="n"/>
+      <c r="M36" s="325" t="n"/>
+      <c r="N36" s="325" t="n"/>
+      <c r="O36" s="325" t="n"/>
+    </row>
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="326" t="inlineStr">
+        <is>
+          <t>Same Drivers tab, frozen 26 Sep 2026, events $40k / quarter on the 2027 rows above. 2026 P1–P10 = Toast actrevs + Cloudbeds bookedrevs (36 keys). P11 = typed uhg-forecast (FP $77k / 1887 $135k / SOCC $29k / rooms $135k). P12 = 2026 36-key file (no typed KV): FP $55k / 1887 $102k / SOCC $19k / rooms 35% × $190 ADR. P13 2026 left blank on purpose. Do not mix P11 open actuals into this row.</t>
+        </is>
+      </c>
+      <c r="B37" s="325" t="n"/>
+      <c r="C37" s="325" t="n"/>
+      <c r="D37" s="325" t="n"/>
+      <c r="E37" s="325" t="n"/>
+      <c r="F37" s="325" t="n"/>
+      <c r="G37" s="325" t="n"/>
+      <c r="H37" s="325" t="n"/>
+      <c r="I37" s="325" t="n"/>
+      <c r="J37" s="325" t="n"/>
+      <c r="K37" s="325" t="n"/>
+      <c r="L37" s="325" t="n"/>
+      <c r="M37" s="325" t="n"/>
+      <c r="N37" s="325" t="n"/>
+      <c r="O37" s="325" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="327" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="B39" s="328" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C39" s="328" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D39" s="328" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E39" s="328" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="F39" s="328" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="G39" s="328" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="H39" s="328" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="I39" s="328" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="J39" s="328" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="K39" s="328" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="L39" s="328" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="M39" s="328" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="N39" s="328" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="O39" s="328" t="inlineStr">
+        <is>
+          <t>P1–P12</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="329" t="inlineStr">
+        <is>
+          <t>2026 source</t>
+        </is>
+      </c>
+      <c r="B40" s="330" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="C40" s="330" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="D40" s="330" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="E40" s="330" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="F40" s="330" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="G40" s="330" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="H40" s="330" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="I40" s="330" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="J40" s="330" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="K40" s="330" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="L40" s="331" t="inlineStr">
+        <is>
+          <t>Forecast</t>
+        </is>
+      </c>
+      <c r="M40" s="331" t="inlineStr">
+        <is>
+          <t>Forecast</t>
+        </is>
+      </c>
+      <c r="N40" s="332" t="n"/>
+      <c r="O40" s="328" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="333" t="inlineStr">
+        <is>
+          <t>2026 Hotel room revenue</t>
+        </is>
+      </c>
+      <c r="B41" s="334" t="n">
+        <v>35707.95</v>
+      </c>
+      <c r="C41" s="334" t="n">
+        <v>50119.63</v>
+      </c>
+      <c r="D41" s="334" t="n">
+        <v>46802.61</v>
+      </c>
+      <c r="E41" s="334" t="n">
+        <v>65355.83</v>
+      </c>
+      <c r="F41" s="334" t="n">
+        <v>72347.02</v>
+      </c>
+      <c r="G41" s="334" t="n">
+        <v>111166.4</v>
+      </c>
+      <c r="H41" s="334" t="n">
+        <v>127586.94</v>
+      </c>
+      <c r="I41" s="334" t="n">
+        <v>133120.04</v>
+      </c>
+      <c r="J41" s="334" t="n">
+        <v>119031.55</v>
+      </c>
+      <c r="K41" s="334" t="n">
+        <v>143720.85</v>
+      </c>
+      <c r="L41" s="335" t="n">
+        <v>135000</v>
+      </c>
+      <c r="M41" s="335" t="n">
+        <v>67032</v>
+      </c>
+      <c r="N41" s="336" t="n"/>
+      <c r="O41" s="337">
+        <f>SUM(B41:M41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="333" t="inlineStr">
+        <is>
+          <t>2026 Fremont Provisions</t>
+        </is>
+      </c>
+      <c r="B42" s="334" t="n">
+        <v>58993.08</v>
+      </c>
+      <c r="C42" s="334" t="n">
+        <v>56760.31</v>
+      </c>
+      <c r="D42" s="334" t="n">
+        <v>59796.12</v>
+      </c>
+      <c r="E42" s="334" t="n">
+        <v>66252.02</v>
+      </c>
+      <c r="F42" s="334" t="n">
+        <v>73080.39999999999</v>
+      </c>
+      <c r="G42" s="334" t="n">
+        <v>74453.69</v>
+      </c>
+      <c r="H42" s="334" t="n">
+        <v>70514.83</v>
+      </c>
+      <c r="I42" s="334" t="n">
+        <v>83752.07000000001</v>
+      </c>
+      <c r="J42" s="334" t="n">
+        <v>76773.3</v>
+      </c>
+      <c r="K42" s="334" t="n">
+        <v>82000.07000000001</v>
+      </c>
+      <c r="L42" s="335" t="n">
+        <v>77000</v>
+      </c>
+      <c r="M42" s="335" t="n">
+        <v>55000</v>
+      </c>
+      <c r="N42" s="336" t="n"/>
+      <c r="O42" s="337">
+        <f>SUM(B42:M42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="333" t="inlineStr">
+        <is>
+          <t>2026 1887 / hotel F&amp;B</t>
+        </is>
+      </c>
+      <c r="B43" s="334" t="n">
+        <v>87790.25999999999</v>
+      </c>
+      <c r="C43" s="334" t="n">
+        <v>109890</v>
+      </c>
+      <c r="D43" s="334" t="n">
+        <v>99423.5</v>
+      </c>
+      <c r="E43" s="334" t="n">
+        <v>113697.29</v>
+      </c>
+      <c r="F43" s="334" t="n">
+        <v>122124.07</v>
+      </c>
+      <c r="G43" s="334" t="n">
+        <v>126190.39</v>
+      </c>
+      <c r="H43" s="334" t="n">
+        <v>134412.89</v>
+      </c>
+      <c r="I43" s="334" t="n">
+        <v>157572.22</v>
+      </c>
+      <c r="J43" s="334" t="n">
+        <v>141680.48</v>
+      </c>
+      <c r="K43" s="334" t="n">
+        <v>145221.77</v>
+      </c>
+      <c r="L43" s="335" t="n">
+        <v>135000</v>
+      </c>
+      <c r="M43" s="335" t="n">
+        <v>102000</v>
+      </c>
+      <c r="N43" s="336" t="n"/>
+      <c r="O43" s="337">
+        <f>SUM(B43:M43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="333" t="inlineStr">
+        <is>
+          <t>2026 Standard Oil</t>
+        </is>
+      </c>
+      <c r="B44" s="334" t="n">
+        <v>16016.19</v>
+      </c>
+      <c r="C44" s="334" t="n">
+        <v>19468.36</v>
+      </c>
+      <c r="D44" s="334" t="n">
+        <v>21187.62</v>
+      </c>
+      <c r="E44" s="334" t="n">
+        <v>24482.84</v>
+      </c>
+      <c r="F44" s="334" t="n">
+        <v>27214.26</v>
+      </c>
+      <c r="G44" s="334" t="n">
+        <v>29759.37</v>
+      </c>
+      <c r="H44" s="334" t="n">
+        <v>31140.71</v>
+      </c>
+      <c r="I44" s="334" t="n">
+        <v>32411.43</v>
+      </c>
+      <c r="J44" s="334" t="n">
+        <v>28860.52</v>
+      </c>
+      <c r="K44" s="334" t="n">
+        <v>30494.13</v>
+      </c>
+      <c r="L44" s="335" t="n">
+        <v>29000</v>
+      </c>
+      <c r="M44" s="335" t="n">
+        <v>19000</v>
+      </c>
+      <c r="N44" s="336" t="n"/>
+      <c r="O44" s="337">
+        <f>SUM(B44:M44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="333" t="inlineStr">
+        <is>
+          <t>2026 Events (actual lumpy)</t>
+        </is>
+      </c>
+      <c r="B45" s="334" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="334" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="334" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="334" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="334" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="334" t="n">
+        <v>47388.61</v>
+      </c>
+      <c r="H45" s="334" t="n">
+        <v>22930.81</v>
+      </c>
+      <c r="I45" s="334" t="n">
+        <v>13693.48</v>
+      </c>
+      <c r="J45" s="334" t="n">
+        <v>17325.82</v>
+      </c>
+      <c r="K45" s="334" t="n">
+        <v>5192.32</v>
+      </c>
+      <c r="L45" s="335" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="335" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" s="336" t="n"/>
+      <c r="O45" s="337">
+        <f>SUM(B45:M45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="338" t="inlineStr">
+        <is>
+          <t>2026 Total F&amp;B + events</t>
+        </is>
+      </c>
+      <c r="B46" s="334">
+        <f>B42+B43+B44+B45</f>
+        <v/>
+      </c>
+      <c r="C46" s="334">
+        <f>C42+C43+C44+C45</f>
+        <v/>
+      </c>
+      <c r="D46" s="334">
+        <f>D42+D43+D44+D45</f>
+        <v/>
+      </c>
+      <c r="E46" s="334">
+        <f>E42+E43+E44+E45</f>
+        <v/>
+      </c>
+      <c r="F46" s="334">
+        <f>F42+F43+F44+F45</f>
+        <v/>
+      </c>
+      <c r="G46" s="334">
+        <f>G42+G43+G44+G45</f>
+        <v/>
+      </c>
+      <c r="H46" s="334">
+        <f>H42+H43+H44+H45</f>
+        <v/>
+      </c>
+      <c r="I46" s="334">
+        <f>I42+I43+I44+I45</f>
+        <v/>
+      </c>
+      <c r="J46" s="334">
+        <f>J42+J43+J44+J45</f>
+        <v/>
+      </c>
+      <c r="K46" s="334">
+        <f>K42+K43+K44+K45</f>
+        <v/>
+      </c>
+      <c r="L46" s="335">
+        <f>L42+L43+L44+L45</f>
+        <v/>
+      </c>
+      <c r="M46" s="335">
+        <f>M42+M43+M44+M45</f>
+        <v/>
+      </c>
+      <c r="N46" s="339" t="n"/>
+      <c r="O46" s="340">
+        <f>SUM(B46:M46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="341" t="inlineStr">
+        <is>
+          <t>2026 TOTAL INCOME</t>
+        </is>
+      </c>
+      <c r="B47" s="340">
+        <f>B41+B46</f>
+        <v/>
+      </c>
+      <c r="C47" s="340">
+        <f>C41+C46</f>
+        <v/>
+      </c>
+      <c r="D47" s="340">
+        <f>D41+D46</f>
+        <v/>
+      </c>
+      <c r="E47" s="340">
+        <f>E41+E46</f>
+        <v/>
+      </c>
+      <c r="F47" s="340">
+        <f>F41+F46</f>
+        <v/>
+      </c>
+      <c r="G47" s="340">
+        <f>G41+G46</f>
+        <v/>
+      </c>
+      <c r="H47" s="340">
+        <f>H41+H46</f>
+        <v/>
+      </c>
+      <c r="I47" s="340">
+        <f>I41+I46</f>
+        <v/>
+      </c>
+      <c r="J47" s="340">
+        <f>J41+J46</f>
+        <v/>
+      </c>
+      <c r="K47" s="340">
+        <f>K41+K46</f>
+        <v/>
+      </c>
+      <c r="L47" s="340">
+        <f>L41+L46</f>
+        <v/>
+      </c>
+      <c r="M47" s="340">
+        <f>M41+M46</f>
+        <v/>
+      </c>
+      <c r="N47" s="342" t="n"/>
+      <c r="O47" s="340">
+        <f>SUM(B47:M47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="341" t="inlineStr">
+        <is>
+          <t>2027 TOTAL INCOME (frozen)</t>
+        </is>
+      </c>
+      <c r="B49" s="340">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="C49" s="340">
+        <f>C17</f>
+        <v/>
+      </c>
+      <c r="D49" s="340">
+        <f>D17</f>
+        <v/>
+      </c>
+      <c r="E49" s="340">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="F49" s="340">
+        <f>F17</f>
+        <v/>
+      </c>
+      <c r="G49" s="340">
+        <f>G17</f>
+        <v/>
+      </c>
+      <c r="H49" s="340">
+        <f>H17</f>
+        <v/>
+      </c>
+      <c r="I49" s="340">
+        <f>I17</f>
+        <v/>
+      </c>
+      <c r="J49" s="340">
+        <f>J17</f>
+        <v/>
+      </c>
+      <c r="K49" s="340">
+        <f>K17</f>
+        <v/>
+      </c>
+      <c r="L49" s="340">
+        <f>L17</f>
+        <v/>
+      </c>
+      <c r="M49" s="340">
+        <f>M17</f>
+        <v/>
+      </c>
+      <c r="N49" s="340">
+        <f>N17</f>
+        <v/>
+      </c>
+      <c r="O49" s="340">
+        <f>SUM(B49:M49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="343" t="inlineStr">
+        <is>
+          <t>$  2027 vs 2026</t>
+        </is>
+      </c>
+      <c r="B50" s="344">
+        <f>B49-B47</f>
+        <v/>
+      </c>
+      <c r="C50" s="344">
+        <f>C49-C47</f>
+        <v/>
+      </c>
+      <c r="D50" s="344">
+        <f>D49-D47</f>
+        <v/>
+      </c>
+      <c r="E50" s="344">
+        <f>E49-E47</f>
+        <v/>
+      </c>
+      <c r="F50" s="344">
+        <f>F49-F47</f>
+        <v/>
+      </c>
+      <c r="G50" s="344">
+        <f>G49-G47</f>
+        <v/>
+      </c>
+      <c r="H50" s="344">
+        <f>H49-H47</f>
+        <v/>
+      </c>
+      <c r="I50" s="344">
+        <f>I49-I47</f>
+        <v/>
+      </c>
+      <c r="J50" s="344">
+        <f>J49-J47</f>
+        <v/>
+      </c>
+      <c r="K50" s="344">
+        <f>K49-K47</f>
+        <v/>
+      </c>
+      <c r="L50" s="344">
+        <f>L49-L47</f>
+        <v/>
+      </c>
+      <c r="M50" s="344">
+        <f>M49-M47</f>
+        <v/>
+      </c>
+      <c r="N50" s="339" t="n"/>
+      <c r="O50" s="345">
+        <f>O49-O47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="343" t="inlineStr">
+        <is>
+          <t>%  2027 vs 2026</t>
+        </is>
+      </c>
+      <c r="B51" s="346">
+        <f>IF(B47=0,"",B50/B47)</f>
+        <v/>
+      </c>
+      <c r="C51" s="346">
+        <f>IF(C47=0,"",C50/C47)</f>
+        <v/>
+      </c>
+      <c r="D51" s="346">
+        <f>IF(D47=0,"",D50/D47)</f>
+        <v/>
+      </c>
+      <c r="E51" s="346">
+        <f>IF(E47=0,"",E50/E47)</f>
+        <v/>
+      </c>
+      <c r="F51" s="346">
+        <f>IF(F47=0,"",F50/F47)</f>
+        <v/>
+      </c>
+      <c r="G51" s="346">
+        <f>IF(G47=0,"",G50/G47)</f>
+        <v/>
+      </c>
+      <c r="H51" s="346">
+        <f>IF(H47=0,"",H50/H47)</f>
+        <v/>
+      </c>
+      <c r="I51" s="346">
+        <f>IF(I47=0,"",I50/I47)</f>
+        <v/>
+      </c>
+      <c r="J51" s="346">
+        <f>IF(J47=0,"",J50/J47)</f>
+        <v/>
+      </c>
+      <c r="K51" s="346">
+        <f>IF(K47=0,"",K50/K47)</f>
+        <v/>
+      </c>
+      <c r="L51" s="346">
+        <f>IF(L47=0,"",L50/L47)</f>
+        <v/>
+      </c>
+      <c r="M51" s="346">
+        <f>IF(M47=0,"",M50/M47)</f>
+        <v/>
+      </c>
+      <c r="N51" s="339" t="n"/>
+      <c r="O51" s="347">
+        <f>IF(O47=0,"",O50/O47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="348" t="inlineStr">
+        <is>
+          <t>Notes on this comparison</t>
+        </is>
+      </c>
+      <c r="B53" s="325" t="n"/>
+      <c r="C53" s="325" t="n"/>
+      <c r="D53" s="325" t="n"/>
+      <c r="E53" s="325" t="n"/>
+      <c r="F53" s="325" t="n"/>
+      <c r="G53" s="325" t="n"/>
+      <c r="H53" s="325" t="n"/>
+      <c r="I53" s="325" t="n"/>
+      <c r="J53" s="325" t="n"/>
+      <c r="K53" s="325" t="n"/>
+      <c r="L53" s="325" t="n"/>
+      <c r="M53" s="325" t="n"/>
+      <c r="N53" s="325" t="n"/>
+      <c r="O53" s="325" t="n"/>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="326" t="inlineStr">
+        <is>
+          <t>1. P1–P10 2026 is posted actuals as of 13 Oct 2026. P10 is closed. P11 is open — do not use the partial Toast week as the 2026 number.</t>
+        </is>
+      </c>
+      <c r="B54" s="325" t="n"/>
+      <c r="C54" s="325" t="n"/>
+      <c r="D54" s="325" t="n"/>
+      <c r="E54" s="325" t="n"/>
+      <c r="F54" s="325" t="n"/>
+      <c r="G54" s="325" t="n"/>
+      <c r="H54" s="325" t="n"/>
+      <c r="I54" s="325" t="n"/>
+      <c r="J54" s="325" t="n"/>
+      <c r="K54" s="325" t="n"/>
+      <c r="L54" s="325" t="n"/>
+      <c r="M54" s="325" t="n"/>
+      <c r="N54" s="325" t="n"/>
+      <c r="O54" s="325" t="n"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="326" t="inlineStr">
+        <is>
+          <t>2. P11 forecast is the typed period budget on the labor summary (uhg-forecast), not the old 75% / $166k hotel line.</t>
+        </is>
+      </c>
+      <c r="B55" s="325" t="n"/>
+      <c r="C55" s="325" t="n"/>
+      <c r="D55" s="325" t="n"/>
+      <c r="E55" s="325" t="n"/>
+      <c r="F55" s="325" t="n"/>
+      <c r="G55" s="325" t="n"/>
+      <c r="H55" s="325" t="n"/>
+      <c r="I55" s="325" t="n"/>
+      <c r="J55" s="325" t="n"/>
+      <c r="K55" s="325" t="n"/>
+      <c r="L55" s="325" t="n"/>
+      <c r="M55" s="325" t="n"/>
+      <c r="N55" s="325" t="n"/>
+      <c r="O55" s="325" t="n"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="326" t="inlineStr">
+        <is>
+          <t>3. P12 forecast is the 2026 36-key COMPANY INCOME STATEMENT file (no typed KV yet). Rooms = 36 × 28 × 35% × $190 = $67,032.</t>
+        </is>
+      </c>
+      <c r="B56" s="325" t="n"/>
+      <c r="C56" s="325" t="n"/>
+      <c r="D56" s="325" t="n"/>
+      <c r="E56" s="325" t="n"/>
+      <c r="F56" s="325" t="n"/>
+      <c r="G56" s="325" t="n"/>
+      <c r="H56" s="325" t="n"/>
+      <c r="I56" s="325" t="n"/>
+      <c r="J56" s="325" t="n"/>
+      <c r="K56" s="325" t="n"/>
+      <c r="L56" s="325" t="n"/>
+      <c r="M56" s="325" t="n"/>
+      <c r="N56" s="325" t="n"/>
+      <c r="O56" s="325" t="n"/>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="326" t="inlineStr">
+        <is>
+          <t>4. 2027 events stay $40k / quarter even. 2026 events are the lumpy actuals (mostly P6–P10). That is the point of the freeze.</t>
+        </is>
+      </c>
+      <c r="B57" s="325" t="n"/>
+      <c r="C57" s="325" t="n"/>
+      <c r="D57" s="325" t="n"/>
+      <c r="E57" s="325" t="n"/>
+      <c r="F57" s="325" t="n"/>
+      <c r="G57" s="325" t="n"/>
+      <c r="H57" s="325" t="n"/>
+      <c r="I57" s="325" t="n"/>
+      <c r="J57" s="325" t="n"/>
+      <c r="K57" s="325" t="n"/>
+      <c r="L57" s="325" t="n"/>
+      <c r="M57" s="325" t="n"/>
+      <c r="N57" s="325" t="n"/>
+      <c r="O57" s="325" t="n"/>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="326" t="inlineStr">
+        <is>
+          <t>5. Column O is P1–P12 only so the two years sit on the same 12 periods. P13 2026 is blank until that forecast is typed.</t>
+        </is>
+      </c>
+      <c r="B58" s="325" t="n"/>
+      <c r="C58" s="325" t="n"/>
+      <c r="D58" s="325" t="n"/>
+      <c r="E58" s="325" t="n"/>
+      <c r="F58" s="325" t="n"/>
+      <c r="G58" s="325" t="n"/>
+      <c r="H58" s="325" t="n"/>
+      <c r="I58" s="325" t="n"/>
+      <c r="J58" s="325" t="n"/>
+      <c r="K58" s="325" t="n"/>
+      <c r="L58" s="325" t="n"/>
+      <c r="M58" s="325" t="n"/>
+      <c r="N58" s="325" t="n"/>
+      <c r="O58" s="325" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="16">
+    <mergeCell ref="A55:O55"/>
     <mergeCell ref="A29:O29"/>
+    <mergeCell ref="A57:O57"/>
     <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A54:O54"/>
     <mergeCell ref="A33:O33"/>
+    <mergeCell ref="A36:O36"/>
     <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A37:O37"/>
     <mergeCell ref="A32:O32"/>
     <mergeCell ref="A31:O31"/>
+    <mergeCell ref="A58:O58"/>
     <mergeCell ref="A34:O34"/>
+    <mergeCell ref="A56:O56"/>
     <mergeCell ref="A30:O30"/>
+    <mergeCell ref="A53:O53"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -3242,7 +4263,7 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B5" s="243" t="n">
+      <c r="B5" s="349" t="n">
         <v>46384</v>
       </c>
       <c r="C5" s="232" t="n">
@@ -3282,7 +4303,7 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B6" s="243" t="n">
+      <c r="B6" s="349" t="n">
         <v>46391</v>
       </c>
       <c r="C6" s="232" t="n">
@@ -3322,7 +4343,7 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B7" s="243" t="n">
+      <c r="B7" s="349" t="n">
         <v>46398</v>
       </c>
       <c r="C7" s="232" t="n">
@@ -3362,7 +4383,7 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="B8" s="245" t="n">
+      <c r="B8" s="350" t="n">
         <v>46405</v>
       </c>
       <c r="C8" s="235" t="n">
@@ -3402,7 +4423,7 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="B9" s="243" t="n">
+      <c r="B9" s="349" t="n">
         <v>46412</v>
       </c>
       <c r="C9" s="232" t="n">
@@ -3442,7 +4463,7 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="B10" s="243" t="n">
+      <c r="B10" s="349" t="n">
         <v>46419</v>
       </c>
       <c r="C10" s="232" t="n">
@@ -3482,7 +4503,7 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="B11" s="243" t="n">
+      <c r="B11" s="349" t="n">
         <v>46426</v>
       </c>
       <c r="C11" s="232" t="n">
@@ -3522,7 +4543,7 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="B12" s="245" t="n">
+      <c r="B12" s="350" t="n">
         <v>46433</v>
       </c>
       <c r="C12" s="235" t="n">
@@ -3562,7 +4583,7 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="B13" s="243" t="n">
+      <c r="B13" s="349" t="n">
         <v>46440</v>
       </c>
       <c r="C13" s="232" t="n">
@@ -3602,7 +4623,7 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="B14" s="243" t="n">
+      <c r="B14" s="349" t="n">
         <v>46447</v>
       </c>
       <c r="C14" s="232" t="n">
@@ -3642,7 +4663,7 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="B15" s="243" t="n">
+      <c r="B15" s="349" t="n">
         <v>46454</v>
       </c>
       <c r="C15" s="232" t="n">
@@ -3682,7 +4703,7 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="B16" s="245" t="n">
+      <c r="B16" s="350" t="n">
         <v>46461</v>
       </c>
       <c r="C16" s="235" t="n">
@@ -3722,7 +4743,7 @@
           <t>P4</t>
         </is>
       </c>
-      <c r="B17" s="243" t="n">
+      <c r="B17" s="349" t="n">
         <v>46468</v>
       </c>
       <c r="C17" s="232" t="n">
@@ -3762,7 +4783,7 @@
           <t>P4</t>
         </is>
       </c>
-      <c r="B18" s="243" t="n">
+      <c r="B18" s="349" t="n">
         <v>46475</v>
       </c>
       <c r="C18" s="232" t="n">
@@ -3802,7 +4823,7 @@
           <t>P4</t>
         </is>
       </c>
-      <c r="B19" s="243" t="n">
+      <c r="B19" s="349" t="n">
         <v>46482</v>
       </c>
       <c r="C19" s="232" t="n">
@@ -3842,7 +4863,7 @@
           <t>P4</t>
         </is>
       </c>
-      <c r="B20" s="245" t="n">
+      <c r="B20" s="350" t="n">
         <v>46489</v>
       </c>
       <c r="C20" s="235" t="n">
@@ -3882,7 +4903,7 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="B21" s="243" t="n">
+      <c r="B21" s="349" t="n">
         <v>46496</v>
       </c>
       <c r="C21" s="232" t="n">
@@ -3922,7 +4943,7 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="B22" s="243" t="n">
+      <c r="B22" s="349" t="n">
         <v>46503</v>
       </c>
       <c r="C22" s="232" t="n">
@@ -3962,7 +4983,7 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="B23" s="243" t="n">
+      <c r="B23" s="349" t="n">
         <v>46510</v>
       </c>
       <c r="C23" s="232" t="n">
@@ -4002,7 +5023,7 @@
           <t>P5</t>
         </is>
       </c>
-      <c r="B24" s="245" t="n">
+      <c r="B24" s="350" t="n">
         <v>46517</v>
       </c>
       <c r="C24" s="235" t="n">
@@ -4042,7 +5063,7 @@
           <t>P6</t>
         </is>
       </c>
-      <c r="B25" s="243" t="n">
+      <c r="B25" s="349" t="n">
         <v>46524</v>
       </c>
       <c r="C25" s="232" t="n">
@@ -4082,7 +5103,7 @@
           <t>P6</t>
         </is>
       </c>
-      <c r="B26" s="243" t="n">
+      <c r="B26" s="349" t="n">
         <v>46531</v>
       </c>
       <c r="C26" s="232" t="n">
@@ -4122,7 +5143,7 @@
           <t>P6</t>
         </is>
       </c>
-      <c r="B27" s="243" t="n">
+      <c r="B27" s="349" t="n">
         <v>46538</v>
       </c>
       <c r="C27" s="232" t="n">
@@ -4162,7 +5183,7 @@
           <t>P6</t>
         </is>
       </c>
-      <c r="B28" s="245" t="n">
+      <c r="B28" s="350" t="n">
         <v>46545</v>
       </c>
       <c r="C28" s="235" t="n">
@@ -4202,7 +5223,7 @@
           <t>P7</t>
         </is>
       </c>
-      <c r="B29" s="243" t="n">
+      <c r="B29" s="349" t="n">
         <v>46552</v>
       </c>
       <c r="C29" s="232" t="n">
@@ -4242,7 +5263,7 @@
           <t>P7</t>
         </is>
       </c>
-      <c r="B30" s="243" t="n">
+      <c r="B30" s="349" t="n">
         <v>46559</v>
       </c>
       <c r="C30" s="232" t="n">
@@ -4282,7 +5303,7 @@
           <t>P7</t>
         </is>
       </c>
-      <c r="B31" s="243" t="n">
+      <c r="B31" s="349" t="n">
         <v>46566</v>
       </c>
       <c r="C31" s="232" t="n">
@@ -4322,7 +5343,7 @@
           <t>P7</t>
         </is>
       </c>
-      <c r="B32" s="245" t="n">
+      <c r="B32" s="350" t="n">
         <v>46573</v>
       </c>
       <c r="C32" s="235" t="n">
@@ -4362,7 +5383,7 @@
           <t>P8</t>
         </is>
       </c>
-      <c r="B33" s="243" t="n">
+      <c r="B33" s="349" t="n">
         <v>46580</v>
       </c>
       <c r="C33" s="232" t="n">
@@ -4402,7 +5423,7 @@
           <t>P8</t>
         </is>
       </c>
-      <c r="B34" s="243" t="n">
+      <c r="B34" s="349" t="n">
         <v>46587</v>
       </c>
       <c r="C34" s="232" t="n">
@@ -4442,7 +5463,7 @@
           <t>P8</t>
         </is>
       </c>
-      <c r="B35" s="243" t="n">
+      <c r="B35" s="349" t="n">
         <v>46594</v>
       </c>
       <c r="C35" s="232" t="n">
@@ -4482,7 +5503,7 @@
           <t>P8</t>
         </is>
       </c>
-      <c r="B36" s="245" t="n">
+      <c r="B36" s="350" t="n">
         <v>46601</v>
       </c>
       <c r="C36" s="235" t="n">
@@ -4522,7 +5543,7 @@
           <t>P9</t>
         </is>
       </c>
-      <c r="B37" s="243" t="n">
+      <c r="B37" s="349" t="n">
         <v>46608</v>
       </c>
       <c r="C37" s="232" t="n">
@@ -4562,7 +5583,7 @@
           <t>P9</t>
         </is>
       </c>
-      <c r="B38" s="243" t="n">
+      <c r="B38" s="349" t="n">
         <v>46615</v>
       </c>
       <c r="C38" s="232" t="n">
@@ -4602,7 +5623,7 @@
           <t>P9</t>
         </is>
       </c>
-      <c r="B39" s="243" t="n">
+      <c r="B39" s="349" t="n">
         <v>46622</v>
       </c>
       <c r="C39" s="232" t="n">
@@ -4642,7 +5663,7 @@
           <t>P9</t>
         </is>
       </c>
-      <c r="B40" s="245" t="n">
+      <c r="B40" s="350" t="n">
         <v>46629</v>
       </c>
       <c r="C40" s="235" t="n">
@@ -4682,7 +5703,7 @@
           <t>P10</t>
         </is>
       </c>
-      <c r="B41" s="243" t="n">
+      <c r="B41" s="349" t="n">
         <v>46636</v>
       </c>
       <c r="C41" s="232" t="n">
@@ -4722,7 +5743,7 @@
           <t>P10</t>
         </is>
       </c>
-      <c r="B42" s="243" t="n">
+      <c r="B42" s="349" t="n">
         <v>46643</v>
       </c>
       <c r="C42" s="232" t="n">
@@ -4762,7 +5783,7 @@
           <t>P10</t>
         </is>
       </c>
-      <c r="B43" s="243" t="n">
+      <c r="B43" s="349" t="n">
         <v>46650</v>
       </c>
       <c r="C43" s="232" t="n">
@@ -4802,7 +5823,7 @@
           <t>P10</t>
         </is>
       </c>
-      <c r="B44" s="245" t="n">
+      <c r="B44" s="350" t="n">
         <v>46657</v>
       </c>
       <c r="C44" s="235" t="n">
@@ -4842,7 +5863,7 @@
           <t>P11</t>
         </is>
       </c>
-      <c r="B45" s="243" t="n">
+      <c r="B45" s="349" t="n">
         <v>46664</v>
       </c>
       <c r="C45" s="232" t="n">
@@ -4882,7 +5903,7 @@
           <t>P11</t>
         </is>
       </c>
-      <c r="B46" s="243" t="n">
+      <c r="B46" s="349" t="n">
         <v>46671</v>
       </c>
       <c r="C46" s="232" t="n">
@@ -4922,7 +5943,7 @@
           <t>P11</t>
         </is>
       </c>
-      <c r="B47" s="243" t="n">
+      <c r="B47" s="349" t="n">
         <v>46678</v>
       </c>
       <c r="C47" s="232" t="n">
@@ -4962,7 +5983,7 @@
           <t>P11</t>
         </is>
       </c>
-      <c r="B48" s="245" t="n">
+      <c r="B48" s="350" t="n">
         <v>46685</v>
       </c>
       <c r="C48" s="235" t="n">
@@ -5002,7 +6023,7 @@
           <t>P12</t>
         </is>
       </c>
-      <c r="B49" s="243" t="n">
+      <c r="B49" s="349" t="n">
         <v>46692</v>
       </c>
       <c r="C49" s="232" t="n">
@@ -5042,7 +6063,7 @@
           <t>P12</t>
         </is>
       </c>
-      <c r="B50" s="243" t="n">
+      <c r="B50" s="349" t="n">
         <v>46699</v>
       </c>
       <c r="C50" s="232" t="n">
@@ -5082,7 +6103,7 @@
           <t>P12</t>
         </is>
       </c>
-      <c r="B51" s="243" t="n">
+      <c r="B51" s="349" t="n">
         <v>46706</v>
       </c>
       <c r="C51" s="232" t="n">
@@ -5122,7 +6143,7 @@
           <t>P12</t>
         </is>
       </c>
-      <c r="B52" s="245" t="n">
+      <c r="B52" s="350" t="n">
         <v>46713</v>
       </c>
       <c r="C52" s="235" t="n">
@@ -5162,7 +6183,7 @@
           <t>P13</t>
         </is>
       </c>
-      <c r="B53" s="243" t="n">
+      <c r="B53" s="349" t="n">
         <v>46720</v>
       </c>
       <c r="C53" s="232" t="n">
@@ -5202,7 +6223,7 @@
           <t>P13</t>
         </is>
       </c>
-      <c r="B54" s="243" t="n">
+      <c r="B54" s="349" t="n">
         <v>46727</v>
       </c>
       <c r="C54" s="232" t="n">
@@ -5242,7 +6263,7 @@
           <t>P13</t>
         </is>
       </c>
-      <c r="B55" s="243" t="n">
+      <c r="B55" s="349" t="n">
         <v>46734</v>
       </c>
       <c r="C55" s="232" t="n">
@@ -5282,7 +6303,7 @@
           <t>P13</t>
         </is>
       </c>
-      <c r="B56" s="245" t="n">
+      <c r="B56" s="350" t="n">
         <v>46741</v>
       </c>
       <c r="C56" s="235" t="n">
@@ -13028,10 +14049,6 @@
       <c r="Z124" s="212" t="n"/>
       <c r="AB124" s="212" t="n"/>
     </row>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
     <row r="129">
       <c r="A129" s="95" t="inlineStr">
         <is>

</xml_diff>